<commit_message>
add XRToolKitEssentials data in analysis
</commit_message>
<xml_diff>
--- a/evaluation/results.xlsx
+++ b/evaluation/results.xlsx
@@ -1,34 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruizhengu/Projects/InteractoBot/evaluation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruizhengu/Projects/XRintTest/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F3D2BD-CA07-AC4F-81BA-0EDC1AC987BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB522E0-81AB-2448-8CBE-8A6F9D27712D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26520" activeTab="1" xr2:uid="{484EE131-55FD-F246-A82E-4E47E236206B}"/>
+    <workbookView xWindow="20" yWindow="680" windowWidth="30240" windowHeight="17300" firstSheet="9" activeTab="15" xr2:uid="{484EE131-55FD-F246-A82E-4E47E236206B}"/>
   </bookViews>
   <sheets>
-    <sheet name="VR Template-InteractoBot" sheetId="1" r:id="rId1"/>
+    <sheet name="VR Template-XRintTest" sheetId="1" r:id="rId1"/>
     <sheet name="VR Template-Random" sheetId="2" r:id="rId2"/>
-    <sheet name="XRI Assets-InteractoBot" sheetId="3" r:id="rId3"/>
+    <sheet name="XRI Assets-XRintTest" sheetId="3" r:id="rId3"/>
     <sheet name="XRI Assets-Random" sheetId="4" r:id="rId4"/>
-    <sheet name="EscapeProto-InteractoBot" sheetId="5" r:id="rId5"/>
+    <sheet name="EscapeProto-XRintTest" sheetId="5" r:id="rId5"/>
     <sheet name="EscapeProto-Random" sheetId="6" r:id="rId6"/>
-    <sheet name="EscapeRoom-InteractoBot" sheetId="9" r:id="rId7"/>
+    <sheet name="EscapeRoom-XRintTest" sheetId="9" r:id="rId7"/>
     <sheet name="EscapeRoom-Random" sheetId="10" r:id="rId8"/>
-    <sheet name="GameJam-InteractoBot" sheetId="7" r:id="rId9"/>
+    <sheet name="GameJam-XRintTest" sheetId="7" r:id="rId9"/>
     <sheet name="GameJam-Random" sheetId="8" r:id="rId10"/>
-    <sheet name="XRI Kit-InteractoBot" sheetId="11" r:id="rId11"/>
+    <sheet name="XRI Kit-XRintTest" sheetId="11" r:id="rId11"/>
     <sheet name="XRI Kit-Random" sheetId="12" r:id="rId12"/>
-    <sheet name="XRI Examples-InteractoBot" sheetId="13" r:id="rId13"/>
+    <sheet name="XRI Examples-XRintTest" sheetId="13" r:id="rId13"/>
     <sheet name="XRI Examples-Random" sheetId="14" r:id="rId14"/>
-    <sheet name="Average-InteractoBot" sheetId="15" r:id="rId15"/>
-    <sheet name="Average-Random" sheetId="16" r:id="rId16"/>
+    <sheet name="XRToolKitEssentials-XRintTest" sheetId="18" r:id="rId15"/>
+    <sheet name="XRToolKitEssentials-Random" sheetId="17" r:id="rId16"/>
+    <sheet name="Average-XRintTest" sheetId="15" r:id="rId17"/>
+    <sheet name="Average-Random" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="114">
   <si>
     <t>Time</t>
   </si>
@@ -381,6 +383,15 @@
   </si>
   <si>
     <t>Tempt 10</t>
+  </si>
+  <si>
+    <t>Socket</t>
+  </si>
+  <si>
+    <t>5/5</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -870,7 +881,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -883,15 +894,12 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5490,6 +5498,1442 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A26EAF4-E68C-F446-9D2F-F0E69D01D413}">
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="12" max="12" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1">
+        <f>AVERAGE(C2:G2)</f>
+        <v>0.8</v>
+      </c>
+      <c r="C2" s="1">
+        <f>8/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="D2" s="1">
+        <f>8/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="E2" s="1">
+        <f>8/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="F2" s="1">
+        <f>8/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="G2" s="1">
+        <f>8/10</f>
+        <v>0.8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="1">
+        <v>40.770000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>60</v>
+      </c>
+      <c r="B3" s="1">
+        <f t="shared" ref="B3:B21" si="0">AVERAGE(C3:G3)</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <f>10/10</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <f>10/10</f>
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <f>10/10</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
+        <f>10/10</f>
+        <v>1</v>
+      </c>
+      <c r="G3" s="1">
+        <f>10/10</f>
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="1">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>90</v>
+      </c>
+      <c r="B4" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="shared" ref="C4:G21" si="1">10/10</f>
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="1">
+        <v>40.71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>120</v>
+      </c>
+      <c r="B5" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="1">
+        <v>40.58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>150</v>
+      </c>
+      <c r="B6" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="1">
+        <v>40.22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>180</v>
+      </c>
+      <c r="B7" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C7" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D7" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" s="1">
+        <f>AVERAGE(N2:N6)</f>
+        <v>40.555999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>210</v>
+      </c>
+      <c r="B8" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C8" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>240</v>
+      </c>
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C9" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>270</v>
+      </c>
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C10" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>300</v>
+      </c>
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>330</v>
+      </c>
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C12" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>360</v>
+      </c>
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C13" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G13" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>390</v>
+      </c>
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D14" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>420</v>
+      </c>
+      <c r="B15" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D15" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G15" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>450</v>
+      </c>
+      <c r="B16" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G16" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>480</v>
+      </c>
+      <c r="B17" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E17" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G17" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>510</v>
+      </c>
+      <c r="B18" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F18" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G18" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>540</v>
+      </c>
+      <c r="B19" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C19" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D19" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E19" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F19" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G19" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>570</v>
+      </c>
+      <c r="B20" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C20" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D20" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E20" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F20" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G20" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>600</v>
+      </c>
+      <c r="B21" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C21" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D21" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E21" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="F21" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G21" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77DBE236-4135-A849-993E-B5A600387A10}">
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1">
+        <f>AVERAGE(C2:G2)</f>
+        <v>3.8461538461538464E-3</v>
+      </c>
+      <c r="C2" s="1">
+        <f t="shared" ref="C2:E4" si="0">0/52</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <f t="shared" ref="F2:F21" si="1">1/52</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G2" s="1">
+        <f t="shared" ref="G2:G21" si="2">0/52</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>60</v>
+      </c>
+      <c r="B3" s="1">
+        <f t="shared" ref="B3:B21" si="3">AVERAGE(C3:G3)</f>
+        <v>3.8461538461538464E-3</v>
+      </c>
+      <c r="C3" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D3" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G3" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>90</v>
+      </c>
+      <c r="B4" s="1">
+        <f t="shared" si="3"/>
+        <v>3.8461538461538464E-3</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>120</v>
+      </c>
+      <c r="B5" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C5" s="1">
+        <f>1/52</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D5" s="1">
+        <f>1/52</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E5" s="1">
+        <f>1/52</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>150</v>
+      </c>
+      <c r="B6" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C6" s="1">
+        <f t="shared" ref="C6:E21" si="4">1/52</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D6" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>180</v>
+      </c>
+      <c r="B7" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C7" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>210</v>
+      </c>
+      <c r="B8" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C8" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>240</v>
+      </c>
+      <c r="B9" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C9" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D9" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>270</v>
+      </c>
+      <c r="B10" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C10" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D10" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>300</v>
+      </c>
+      <c r="B11" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C11" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D11" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>330</v>
+      </c>
+      <c r="B12" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C12" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D12" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G12" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>360</v>
+      </c>
+      <c r="B13" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C13" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D13" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G13" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>390</v>
+      </c>
+      <c r="B14" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C14" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D14" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>420</v>
+      </c>
+      <c r="B15" s="1">
+        <f t="shared" si="3"/>
+        <v>1.5384615384615385E-2</v>
+      </c>
+      <c r="C15" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D15" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="F15" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G15" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>450</v>
+      </c>
+      <c r="B16" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C16" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E16" s="1">
+        <f>2/52</f>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G16" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>480</v>
+      </c>
+      <c r="B17" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C17" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D17" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E17" s="1">
+        <f t="shared" ref="E17:E21" si="5">2/52</f>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F17" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G17" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>510</v>
+      </c>
+      <c r="B18" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C18" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D18" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E18" s="1">
+        <f t="shared" si="5"/>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F18" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G18" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>540</v>
+      </c>
+      <c r="B19" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C19" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D19" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E19" s="1">
+        <f t="shared" si="5"/>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F19" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G19" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>570</v>
+      </c>
+      <c r="B20" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C20" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D20" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E20" s="1">
+        <f t="shared" si="5"/>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F20" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G20" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>600</v>
+      </c>
+      <c r="B21" s="1">
+        <f t="shared" si="3"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="C21" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="D21" s="1">
+        <f t="shared" si="4"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E21" s="1">
+        <f t="shared" si="5"/>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="F21" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="G21" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E49D7EB-C7D2-824A-8D7A-8EA3762D7E06}">
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5510,14 +6954,14 @@
         <v>30</v>
       </c>
       <c r="B2" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B2, 'XRI Assets-InteractoBot'!B2, 'EscapeProto-InteractoBot'!B2, 'EscapeRoom-InteractoBot'!B2, 'GameJam-InteractoBot'!B2, 'XRI Kit-InteractoBot'!B2, 'XRI Examples-InteractoBot'!B2)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B2, 'XRI Assets-XRintTest'!B2, 'EscapeProto-XRintTest'!B2, 'EscapeRoom-XRintTest'!B2, 'GameJam-XRintTest'!B2, 'XRI Kit-XRintTest'!B2, 'XRI Examples-XRintTest'!B2)</f>
         <v>0.43009606846725462</v>
       </c>
       <c r="D2" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!M7, 'XRI Assets-InteractoBot'!M7, 'EscapeProto-InteractoBot'!M7, 'EscapeRoom-InteractoBot'!M7, 'GameJam-InteractoBot'!M7, 'XRI Kit-InteractoBot'!M7, 'XRI Examples-InteractoBot'!M7)</f>
+        <f>AVERAGE('VR Template-XRintTest'!M7, 'XRI Assets-XRintTest'!M7, 'EscapeProto-XRintTest'!M7, 'EscapeRoom-XRintTest'!M7, 'GameJam-XRintTest'!M7, 'XRI Kit-XRintTest'!M7, 'XRI Examples-XRintTest'!M7)</f>
         <v>148.21142857142857</v>
       </c>
     </row>
@@ -5526,7 +6970,7 @@
         <v>60</v>
       </c>
       <c r="B3" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B3, 'XRI Assets-InteractoBot'!B3, 'EscapeProto-InteractoBot'!B3, 'EscapeRoom-InteractoBot'!B3, 'GameJam-InteractoBot'!B3, 'XRI Kit-InteractoBot'!B3, 'XRI Examples-InteractoBot'!B3)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B3, 'XRI Assets-XRintTest'!B3, 'EscapeProto-XRintTest'!B3, 'EscapeRoom-XRintTest'!B3, 'GameJam-XRintTest'!B3, 'XRI Kit-XRintTest'!B3, 'XRI Examples-XRintTest'!B3)</f>
         <v>0.65378651414207867</v>
       </c>
     </row>
@@ -5535,7 +6979,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B4, 'XRI Assets-InteractoBot'!B4, 'EscapeProto-InteractoBot'!B4, 'EscapeRoom-InteractoBot'!B4, 'GameJam-InteractoBot'!B4, 'XRI Kit-InteractoBot'!B4, 'XRI Examples-InteractoBot'!B4)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B4, 'XRI Assets-XRintTest'!B4, 'EscapeProto-XRintTest'!B4, 'EscapeRoom-XRintTest'!B4, 'GameJam-XRintTest'!B4, 'XRI Kit-XRintTest'!B4, 'XRI Examples-XRintTest'!B4)</f>
         <v>0.73980481150027155</v>
       </c>
     </row>
@@ -5544,7 +6988,7 @@
         <v>120</v>
       </c>
       <c r="B5" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B5, 'XRI Assets-InteractoBot'!B5, 'EscapeProto-InteractoBot'!B5, 'EscapeRoom-InteractoBot'!B5, 'GameJam-InteractoBot'!B5, 'XRI Kit-InteractoBot'!B5, 'XRI Examples-InteractoBot'!B5)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B5, 'XRI Assets-XRintTest'!B5, 'EscapeProto-XRintTest'!B5, 'EscapeRoom-XRintTest'!B5, 'GameJam-XRintTest'!B5, 'XRI Kit-XRintTest'!B5, 'XRI Examples-XRintTest'!B5)</f>
         <v>0.80542121598770855</v>
       </c>
     </row>
@@ -5553,7 +6997,7 @@
         <v>150</v>
       </c>
       <c r="B6" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B6, 'XRI Assets-InteractoBot'!B6, 'EscapeProto-InteractoBot'!B6, 'EscapeRoom-InteractoBot'!B6, 'GameJam-InteractoBot'!B6, 'XRI Kit-InteractoBot'!B6, 'XRI Examples-InteractoBot'!B6)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B6, 'XRI Assets-XRintTest'!B6, 'EscapeProto-XRintTest'!B6, 'EscapeRoom-XRintTest'!B6, 'GameJam-XRintTest'!B6, 'XRI Kit-XRintTest'!B6, 'XRI Examples-XRintTest'!B6)</f>
         <v>0.85228875182671893</v>
       </c>
     </row>
@@ -5562,7 +7006,7 @@
         <v>180</v>
       </c>
       <c r="B7" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B7, 'XRI Assets-InteractoBot'!B7, 'EscapeProto-InteractoBot'!B7, 'EscapeRoom-InteractoBot'!B7, 'GameJam-InteractoBot'!B7, 'XRI Kit-InteractoBot'!B7, 'XRI Examples-InteractoBot'!B7)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B7, 'XRI Assets-XRintTest'!B7, 'EscapeProto-XRintTest'!B7, 'EscapeRoom-XRintTest'!B7, 'GameJam-XRintTest'!B7, 'XRI Kit-XRintTest'!B7, 'XRI Examples-XRintTest'!B7)</f>
         <v>0.87738312310429634</v>
       </c>
     </row>
@@ -5571,7 +7015,7 @@
         <v>210</v>
       </c>
       <c r="B8" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B8, 'XRI Assets-InteractoBot'!B8, 'EscapeProto-InteractoBot'!B8, 'EscapeRoom-InteractoBot'!B8, 'GameJam-InteractoBot'!B8, 'XRI Kit-InteractoBot'!B8, 'XRI Examples-InteractoBot'!B8)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B8, 'XRI Assets-XRintTest'!B8, 'EscapeProto-XRintTest'!B8, 'EscapeRoom-XRintTest'!B8, 'GameJam-XRintTest'!B8, 'XRI Kit-XRintTest'!B8, 'XRI Examples-XRintTest'!B8)</f>
         <v>0.90490178764586149</v>
       </c>
     </row>
@@ -5580,7 +7024,7 @@
         <v>240</v>
       </c>
       <c r="B9" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B9, 'XRI Assets-InteractoBot'!B9, 'EscapeProto-InteractoBot'!B9, 'EscapeRoom-InteractoBot'!B9, 'GameJam-InteractoBot'!B9, 'XRI Kit-InteractoBot'!B9, 'XRI Examples-InteractoBot'!B9)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B9, 'XRI Assets-XRintTest'!B9, 'EscapeProto-XRintTest'!B9, 'EscapeRoom-XRintTest'!B9, 'GameJam-XRintTest'!B9, 'XRI Kit-XRintTest'!B9, 'XRI Examples-XRintTest'!B9)</f>
         <v>0.92230385123113134</v>
       </c>
     </row>
@@ -5589,7 +7033,7 @@
         <v>270</v>
       </c>
       <c r="B10" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B10, 'XRI Assets-InteractoBot'!B10, 'EscapeProto-InteractoBot'!B10, 'EscapeRoom-InteractoBot'!B10, 'GameJam-InteractoBot'!B10, 'XRI Kit-InteractoBot'!B10, 'XRI Examples-InteractoBot'!B10)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B10, 'XRI Assets-XRintTest'!B10, 'EscapeProto-XRintTest'!B10, 'EscapeRoom-XRintTest'!B10, 'GameJam-XRintTest'!B10, 'XRI Kit-XRintTest'!B10, 'XRI Examples-XRintTest'!B10)</f>
         <v>0.93255466911553697</v>
       </c>
     </row>
@@ -5598,7 +7042,7 @@
         <v>300</v>
       </c>
       <c r="B11" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B11, 'XRI Assets-InteractoBot'!B11, 'EscapeProto-InteractoBot'!B11, 'EscapeRoom-InteractoBot'!B11, 'GameJam-InteractoBot'!B11, 'XRI Kit-InteractoBot'!B11, 'XRI Examples-InteractoBot'!B11)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B11, 'XRI Assets-XRintTest'!B11, 'EscapeProto-XRintTest'!B11, 'EscapeRoom-XRintTest'!B11, 'GameJam-XRintTest'!B11, 'XRI Kit-XRintTest'!B11, 'XRI Examples-XRintTest'!B11)</f>
         <v>0.94302358950812148</v>
       </c>
     </row>
@@ -5607,7 +7051,7 @@
         <v>330</v>
       </c>
       <c r="B12" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B12, 'XRI Assets-InteractoBot'!B12, 'EscapeProto-InteractoBot'!B12, 'EscapeRoom-InteractoBot'!B12, 'GameJam-InteractoBot'!B12, 'XRI Kit-InteractoBot'!B12, 'XRI Examples-InteractoBot'!B12)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B12, 'XRI Assets-XRintTest'!B12, 'EscapeProto-XRintTest'!B12, 'EscapeRoom-XRintTest'!B12, 'GameJam-XRintTest'!B12, 'XRI Kit-XRintTest'!B12, 'XRI Examples-XRintTest'!B12)</f>
         <v>0.95392871491706366</v>
       </c>
     </row>
@@ -5616,7 +7060,7 @@
         <v>360</v>
       </c>
       <c r="B13" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B13, 'XRI Assets-InteractoBot'!B13, 'EscapeProto-InteractoBot'!B13, 'EscapeRoom-InteractoBot'!B13, 'GameJam-InteractoBot'!B13, 'XRI Kit-InteractoBot'!B13, 'XRI Examples-InteractoBot'!B13)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B13, 'XRI Assets-XRintTest'!B13, 'EscapeProto-XRintTest'!B13, 'EscapeRoom-XRintTest'!B13, 'GameJam-XRintTest'!B13, 'XRI Kit-XRintTest'!B13, 'XRI Examples-XRintTest'!B13)</f>
         <v>0.96199850771968087</v>
       </c>
     </row>
@@ -5625,7 +7069,7 @@
         <v>390</v>
       </c>
       <c r="B14" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B14, 'XRI Assets-InteractoBot'!B14, 'EscapeProto-InteractoBot'!B14, 'EscapeRoom-InteractoBot'!B14, 'GameJam-InteractoBot'!B14, 'XRI Kit-InteractoBot'!B14, 'XRI Examples-InteractoBot'!B14)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B14, 'XRI Assets-XRintTest'!B14, 'EscapeProto-XRintTest'!B14, 'EscapeRoom-XRintTest'!B14, 'GameJam-XRintTest'!B14, 'XRI Kit-XRintTest'!B14, 'XRI Examples-XRintTest'!B14)</f>
         <v>0.97094071055501352</v>
       </c>
     </row>
@@ -5634,7 +7078,7 @@
         <v>420</v>
       </c>
       <c r="B15" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B15, 'XRI Assets-InteractoBot'!B15, 'EscapeProto-InteractoBot'!B15, 'EscapeRoom-InteractoBot'!B15, 'GameJam-InteractoBot'!B15, 'XRI Kit-InteractoBot'!B15, 'XRI Examples-InteractoBot'!B15)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B15, 'XRI Assets-XRintTest'!B15, 'EscapeProto-XRintTest'!B15, 'EscapeRoom-XRintTest'!B15, 'GameJam-XRintTest'!B15, 'XRI Kit-XRintTest'!B15, 'XRI Examples-XRintTest'!B15)</f>
         <v>0.98075532342306138</v>
       </c>
     </row>
@@ -5643,7 +7087,7 @@
         <v>450</v>
       </c>
       <c r="B16" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B16, 'XRI Assets-InteractoBot'!B16, 'EscapeProto-InteractoBot'!B16, 'EscapeRoom-InteractoBot'!B16, 'GameJam-InteractoBot'!B16, 'XRI Kit-InteractoBot'!B16, 'XRI Examples-InteractoBot'!B16)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B16, 'XRI Assets-XRintTest'!B16, 'EscapeProto-XRintTest'!B16, 'EscapeRoom-XRintTest'!B16, 'GameJam-XRintTest'!B16, 'XRI Kit-XRintTest'!B16, 'XRI Examples-XRintTest'!B16)</f>
         <v>0.9864259886357114</v>
       </c>
     </row>
@@ -5652,7 +7096,7 @@
         <v>480</v>
       </c>
       <c r="B17" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B17, 'XRI Assets-InteractoBot'!B17, 'EscapeProto-InteractoBot'!B17, 'EscapeRoom-InteractoBot'!B17, 'GameJam-InteractoBot'!B17, 'XRI Kit-InteractoBot'!B17, 'XRI Examples-InteractoBot'!B17)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B17, 'XRI Assets-XRintTest'!B17, 'EscapeProto-XRintTest'!B17, 'EscapeRoom-XRintTest'!B17, 'GameJam-XRintTest'!B17, 'XRI Kit-XRintTest'!B17, 'XRI Examples-XRintTest'!B17)</f>
         <v>0.99013373127475179</v>
       </c>
     </row>
@@ -5661,7 +7105,7 @@
         <v>510</v>
       </c>
       <c r="B18" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B18, 'XRI Assets-InteractoBot'!B18, 'EscapeProto-InteractoBot'!B18, 'EscapeRoom-InteractoBot'!B18, 'GameJam-InteractoBot'!B18, 'XRI Kit-InteractoBot'!B18, 'XRI Examples-InteractoBot'!B18)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B18, 'XRI Assets-XRintTest'!B18, 'EscapeProto-XRintTest'!B18, 'EscapeRoom-XRintTest'!B18, 'GameJam-XRintTest'!B18, 'XRI Kit-XRintTest'!B18, 'XRI Examples-XRintTest'!B18)</f>
         <v>0.99078803879928834</v>
       </c>
     </row>
@@ -5670,7 +7114,7 @@
         <v>540</v>
       </c>
       <c r="B19" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B19, 'XRI Assets-InteractoBot'!B19, 'EscapeProto-InteractoBot'!B19, 'EscapeRoom-InteractoBot'!B19, 'GameJam-InteractoBot'!B19, 'XRI Kit-InteractoBot'!B19, 'XRI Examples-InteractoBot'!B19)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B19, 'XRI Assets-XRintTest'!B19, 'EscapeProto-XRintTest'!B19, 'EscapeRoom-XRintTest'!B19, 'GameJam-XRintTest'!B19, 'XRI Kit-XRintTest'!B19, 'XRI Examples-XRintTest'!B19)</f>
         <v>0.99100614130746723</v>
       </c>
     </row>
@@ -5679,7 +7123,7 @@
         <v>570</v>
       </c>
       <c r="B20" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B20, 'XRI Assets-InteractoBot'!B20, 'EscapeProto-InteractoBot'!B20, 'EscapeRoom-InteractoBot'!B20, 'GameJam-InteractoBot'!B20, 'XRI Kit-InteractoBot'!B20, 'XRI Examples-InteractoBot'!B20)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B20, 'XRI Assets-XRintTest'!B20, 'EscapeProto-XRintTest'!B20, 'EscapeRoom-XRintTest'!B20, 'GameJam-XRintTest'!B20, 'XRI Kit-XRintTest'!B20, 'XRI Examples-XRintTest'!B20)</f>
         <v>0.99100614130746723</v>
       </c>
     </row>
@@ -5688,7 +7132,7 @@
         <v>600</v>
       </c>
       <c r="B21" s="1">
-        <f>AVERAGE('VR Template-InteractoBot'!B21, 'XRI Assets-InteractoBot'!B21, 'EscapeProto-InteractoBot'!B21, 'EscapeRoom-InteractoBot'!B21, 'GameJam-InteractoBot'!B21, 'XRI Kit-InteractoBot'!B21, 'XRI Examples-InteractoBot'!B21)</f>
+        <f>AVERAGE('VR Template-XRintTest'!B21, 'XRI Assets-XRintTest'!B21, 'EscapeProto-XRintTest'!B21, 'EscapeRoom-XRintTest'!B21, 'GameJam-XRintTest'!B21, 'XRI Kit-XRintTest'!B21, 'XRI Examples-XRintTest'!B21)</f>
         <v>0.99100614130746723</v>
       </c>
     </row>
@@ -5697,7 +7141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A06ECB-BB76-6147-8DB0-5BA023E66B2D}">
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5901,7 +7345,6 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="13" width="10.83203125" style="1"/>
-    <col min="14" max="17" width="10.83203125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
@@ -5941,14 +7384,14 @@
       <c r="L1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6" t="s">
+      <c r="N1" s="2"/>
+      <c r="O1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -5985,7 +7428,7 @@
         <v>0.22222222222222221</v>
       </c>
       <c r="I2" s="1">
-        <f>0/9</f>
+        <f t="shared" ref="I2:I7" si="1">0/9</f>
         <v>0</v>
       </c>
       <c r="J2" s="1">
@@ -6000,16 +7443,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N2" t="s">
         <v>103</v>
       </c>
-      <c r="O2" s="9">
-        <v>1</v>
-      </c>
-      <c r="P2" s="9">
+      <c r="O2" s="7">
+        <v>1</v>
+      </c>
+      <c r="P2" s="7">
         <v>8</v>
       </c>
-      <c r="Q2" s="9">
+      <c r="Q2" s="7">
         <v>9</v>
       </c>
     </row>
@@ -6018,7 +7461,7 @@
         <v>60</v>
       </c>
       <c r="B3" s="1">
-        <f t="shared" ref="B3:B21" si="1">AVERAGE(C3:G3)</f>
+        <f t="shared" ref="B3:B21" si="2">AVERAGE(C3:G3)</f>
         <v>0.11111111111111112</v>
       </c>
       <c r="C3" s="1">
@@ -6034,11 +7477,11 @@
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <f t="shared" ref="F3:F8" si="2">2/9</f>
+        <f t="shared" ref="F3:F8" si="3">2/9</f>
         <v>0.22222222222222221</v>
       </c>
       <c r="G3" s="1">
-        <f t="shared" ref="G3:G21" si="3">3/9</f>
+        <f t="shared" ref="G3:G21" si="4">3/9</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="H3" s="1">
@@ -6046,11 +7489,11 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="I3" s="1">
-        <f>0/9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J3" s="1">
-        <f>2/9</f>
+        <f t="shared" ref="J3:J12" si="5">2/9</f>
         <v>0.22222222222222221</v>
       </c>
       <c r="K3" s="1">
@@ -6061,16 +7504,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O3" s="9">
-        <v>0</v>
-      </c>
-      <c r="P3" s="9">
+      <c r="O3" s="7">
+        <v>0</v>
+      </c>
+      <c r="P3" s="7">
         <v>2</v>
       </c>
-      <c r="Q3" s="9">
+      <c r="Q3" s="7">
         <v>2</v>
       </c>
     </row>
@@ -6079,7 +7522,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.17777777777777776</v>
       </c>
       <c r="C4" s="1">
@@ -6095,11 +7538,11 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F4" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="G4" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H4" s="1">
@@ -6107,11 +7550,11 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="I4" s="1">
-        <f>0/9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J4" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K4" s="1">
@@ -6122,16 +7565,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="9">
-        <v>0</v>
-      </c>
-      <c r="P4" s="9">
+      <c r="O4" s="7">
+        <v>0</v>
+      </c>
+      <c r="P4" s="7">
         <v>4</v>
       </c>
-      <c r="Q4" s="9">
+      <c r="Q4" s="7">
         <v>4</v>
       </c>
     </row>
@@ -6140,7 +7583,7 @@
         <v>120</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.24444444444444446</v>
       </c>
       <c r="C5" s="1">
@@ -6156,11 +7599,11 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F5" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="G5" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H5" s="1">
@@ -6168,11 +7611,11 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="I5" s="1">
-        <f>0/9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J5" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K5" s="1">
@@ -6183,16 +7626,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="9">
-        <v>0</v>
-      </c>
-      <c r="P5" s="9">
+      <c r="O5" s="7">
+        <v>0</v>
+      </c>
+      <c r="P5" s="7">
         <v>4</v>
       </c>
-      <c r="Q5" s="9">
+      <c r="Q5" s="7">
         <v>4</v>
       </c>
     </row>
@@ -6201,7 +7644,7 @@
         <v>150</v>
       </c>
       <c r="B6" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.24444444444444446</v>
       </c>
       <c r="C6" s="1">
@@ -6209,7 +7652,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="D6" s="1">
-        <f t="shared" ref="D6:F21" si="4">4/9</f>
+        <f t="shared" ref="D6:F21" si="6">4/9</f>
         <v>0.44444444444444442</v>
       </c>
       <c r="E6" s="1">
@@ -6217,11 +7660,11 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F6" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="G6" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H6" s="1">
@@ -6229,11 +7672,11 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="I6" s="1">
-        <f>0/9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J6" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K6" s="1">
@@ -6244,16 +7687,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="O6" s="9">
-        <v>0</v>
-      </c>
-      <c r="P6" s="9">
+      <c r="O6" s="7">
+        <v>0</v>
+      </c>
+      <c r="P6" s="7">
         <v>5</v>
       </c>
-      <c r="Q6" s="9">
+      <c r="Q6" s="7">
         <v>5</v>
       </c>
     </row>
@@ -6262,15 +7705,15 @@
         <v>180</v>
       </c>
       <c r="B7" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.26666666666666666</v>
       </c>
       <c r="C7" s="1">
-        <f t="shared" ref="C7:C21" si="5">2/9</f>
+        <f t="shared" ref="C7:C21" si="7">2/9</f>
         <v>0.22222222222222221</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E7" s="1">
@@ -6278,11 +7721,11 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F7" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="G7" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H7" s="1">
@@ -6290,11 +7733,11 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="I7" s="1">
-        <f>0/9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J7" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K7" s="1">
@@ -6305,16 +7748,16 @@
         <f>2/9</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O7" s="9">
-        <v>0</v>
-      </c>
-      <c r="P7" s="9">
+      <c r="O7" s="7">
+        <v>0</v>
+      </c>
+      <c r="P7" s="7">
         <v>3</v>
       </c>
-      <c r="Q7" s="9">
+      <c r="Q7" s="7">
         <v>3</v>
       </c>
     </row>
@@ -6323,15 +7766,15 @@
         <v>210</v>
       </c>
       <c r="B8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.26666666666666666</v>
       </c>
       <c r="C8" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D8" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E8" s="1">
@@ -6339,11 +7782,11 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="F8" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="G8" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H8" s="1">
@@ -6355,7 +7798,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="J8" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K8" s="1">
@@ -6366,16 +7809,16 @@
         <f>3/9</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="O8" s="10">
-        <v>0</v>
-      </c>
-      <c r="P8" s="10">
+      <c r="O8" s="1">
+        <v>0</v>
+      </c>
+      <c r="P8" s="1">
         <v>5</v>
       </c>
-      <c r="Q8" s="10">
+      <c r="Q8" s="1">
         <v>5</v>
       </c>
     </row>
@@ -6384,15 +7827,15 @@
         <v>240</v>
       </c>
       <c r="B9" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.31111111111111106</v>
       </c>
       <c r="C9" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D9" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E9" s="1">
@@ -6400,11 +7843,11 @@
         <v>0.22222222222222221</v>
       </c>
       <c r="F9" s="1">
-        <f t="shared" ref="F9:F14" si="6">3/9</f>
+        <f t="shared" ref="F9:F14" si="8">3/9</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H9" s="1">
@@ -6416,27 +7859,27 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="J9" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K9" s="1">
-        <f t="shared" ref="J9:K21" si="7">6/9</f>
+        <f t="shared" ref="J9:K21" si="9">6/9</f>
         <v>0.66666666666666663</v>
       </c>
       <c r="L9" s="1">
         <f>4/9</f>
         <v>0.44444444444444442</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="O9" s="10">
-        <v>0</v>
-      </c>
-      <c r="P9" s="10">
+      <c r="O9" s="1">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1">
         <v>3</v>
       </c>
-      <c r="Q9" s="10">
+      <c r="Q9" s="1">
         <v>3</v>
       </c>
     </row>
@@ -6445,15 +7888,15 @@
         <v>270</v>
       </c>
       <c r="B10" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.31111111111111106</v>
       </c>
       <c r="C10" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E10" s="1">
@@ -6461,15 +7904,15 @@
         <v>0.22222222222222221</v>
       </c>
       <c r="F10" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="G10" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H10" s="1">
-        <f t="shared" ref="H10:J21" si="8">5/9</f>
+        <f t="shared" ref="H10:J21" si="10">5/9</f>
         <v>0.55555555555555558</v>
       </c>
       <c r="I10" s="1">
@@ -6477,27 +7920,27 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="J10" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K10" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L10" s="1">
-        <f t="shared" ref="L10:L21" si="9">4/9</f>
+        <f t="shared" ref="L10:L21" si="11">4/9</f>
         <v>0.44444444444444442</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="O10" s="10">
-        <v>0</v>
-      </c>
-      <c r="P10" s="10">
+      <c r="O10" s="1">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1">
         <v>6</v>
       </c>
-      <c r="Q10" s="10">
+      <c r="Q10" s="1">
         <v>6</v>
       </c>
     </row>
@@ -6506,15 +7949,15 @@
         <v>300</v>
       </c>
       <c r="B11" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="C11" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D11" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E11" s="1">
@@ -6522,15 +7965,15 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="F11" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="G11" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H11" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I11" s="1">
@@ -6538,27 +7981,27 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="J11" s="1">
-        <f>2/9</f>
+        <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="K11" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L11" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
-      <c r="N11" s="6" t="s">
+      <c r="N11" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O11" s="10">
-        <v>0</v>
-      </c>
-      <c r="P11" s="10">
+      <c r="O11" s="1">
+        <v>0</v>
+      </c>
+      <c r="P11" s="1">
         <v>6</v>
       </c>
-      <c r="Q11" s="10">
+      <c r="Q11" s="1">
         <v>6</v>
       </c>
     </row>
@@ -6567,59 +8010,59 @@
         <v>330</v>
       </c>
       <c r="B12" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.35555555555555551</v>
       </c>
       <c r="C12" s="1">
+        <f t="shared" si="7"/>
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="D12" s="1">
+        <f t="shared" si="6"/>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="6"/>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="8"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G12" s="1">
+        <f t="shared" si="4"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="H12" s="1">
+        <f t="shared" si="10"/>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="I12" s="1">
+        <f t="shared" ref="I12:I19" si="12">2/9</f>
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="J12" s="1">
         <f t="shared" si="5"/>
         <v>0.22222222222222221</v>
       </c>
-      <c r="D12" s="1">
-        <f t="shared" si="4"/>
+      <c r="K12" s="1">
+        <f t="shared" si="9"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="L12" s="1">
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
-      <c r="E12" s="1">
-        <f t="shared" si="4"/>
-        <v>0.44444444444444442</v>
-      </c>
-      <c r="F12" s="1">
-        <f t="shared" si="6"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="G12" s="1">
-        <f t="shared" si="3"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="H12" s="1">
-        <f t="shared" si="8"/>
-        <v>0.55555555555555558</v>
-      </c>
-      <c r="I12" s="1">
-        <f>2/9</f>
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="J12" s="1">
-        <f>2/9</f>
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="K12" s="1">
-        <f t="shared" si="7"/>
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="L12" s="1">
-        <f t="shared" si="9"/>
-        <v>0.44444444444444442</v>
-      </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O12" s="10">
-        <v>0</v>
-      </c>
-      <c r="P12" s="10">
+      <c r="O12" s="1">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
         <v>4</v>
       </c>
-      <c r="Q12" s="10">
+      <c r="Q12" s="1">
         <v>4</v>
       </c>
     </row>
@@ -6628,35 +8071,35 @@
         <v>360</v>
       </c>
       <c r="B13" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.35555555555555551</v>
       </c>
       <c r="C13" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D13" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F13" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="G13" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H13" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I13" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J13" s="1">
@@ -6664,25 +8107,25 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="K13" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
-      <c r="N13" s="6" t="s">
+      <c r="N13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O13" s="9">
+      <c r="O13" s="7">
         <f>AVERAGE(O3:O12)</f>
         <v>0</v>
       </c>
-      <c r="P13" s="9">
+      <c r="P13" s="7">
         <f>AVERAGE(P3:P12)</f>
         <v>4.2</v>
       </c>
-      <c r="Q13" s="9">
+      <c r="Q13" s="7">
         <f>AVERAGE(Q3:Q12)</f>
         <v>4.2</v>
       </c>
@@ -6692,35 +8135,35 @@
         <v>390</v>
       </c>
       <c r="B14" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.35555555555555551</v>
       </c>
       <c r="C14" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D14" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F14" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="G14" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H14" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I14" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J14" s="1">
@@ -6728,20 +8171,20 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="K14" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L14" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
-      <c r="O14" s="8" t="s">
+      <c r="O14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P14" s="8" t="s">
+      <c r="P14" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="Q14" s="8" t="s">
+      <c r="Q14" s="6" t="s">
         <v>105</v>
       </c>
     </row>
@@ -6750,35 +8193,35 @@
         <v>420</v>
       </c>
       <c r="B15" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C15" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D15" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F15" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G15" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H15" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I15" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J15" s="1">
@@ -6786,11 +8229,11 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="K15" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L15" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -6799,47 +8242,47 @@
         <v>450</v>
       </c>
       <c r="B16" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C16" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D16" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E16" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F16" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G16" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H16" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I16" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J16" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="K16" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -6848,47 +8291,47 @@
         <v>480</v>
       </c>
       <c r="B17" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C17" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D17" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E17" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F17" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G17" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H17" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I17" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J17" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="K17" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L17" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -6897,47 +8340,47 @@
         <v>510</v>
       </c>
       <c r="B18" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C18" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G18" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I18" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J18" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L18" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -6946,47 +8389,47 @@
         <v>540</v>
       </c>
       <c r="B19" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C19" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D19" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E19" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F19" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G19" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H19" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I19" s="1">
-        <f>2/9</f>
+        <f t="shared" si="12"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="J19" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="K19" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L19" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -6995,31 +8438,31 @@
         <v>570</v>
       </c>
       <c r="B20" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37777777777777777</v>
       </c>
       <c r="C20" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D20" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F20" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="G20" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H20" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I20" s="1">
@@ -7027,15 +8470,15 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="J20" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="K20" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L20" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>
@@ -7044,19 +8487,19 @@
         <v>600</v>
       </c>
       <c r="B21" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
       <c r="C21" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.22222222222222221</v>
       </c>
       <c r="D21" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="E21" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.44444444444444442</v>
       </c>
       <c r="F21" s="1">
@@ -7064,11 +8507,11 @@
         <v>0.55555555555555558</v>
       </c>
       <c r="G21" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H21" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.55555555555555558</v>
       </c>
       <c r="I21" s="1">
@@ -7076,15 +8519,15 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="J21" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="K21" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="L21" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.44444444444444442</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add XRToolKitEssentials random results
</commit_message>
<xml_diff>
--- a/evaluation/results.xlsx
+++ b/evaluation/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruizhengu/Projects/XRintTest/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB522E0-81AB-2448-8CBE-8A6F9D27712D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD767B5-5B21-9C43-B142-F24517C50BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="680" windowWidth="30240" windowHeight="17300" firstSheet="9" activeTab="15" xr2:uid="{484EE131-55FD-F246-A82E-4E47E236206B}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17300" firstSheet="9" activeTab="15" xr2:uid="{484EE131-55FD-F246-A82E-4E47E236206B}"/>
   </bookViews>
   <sheets>
     <sheet name="VR Template-XRintTest" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="121">
   <si>
     <t>Time</t>
   </si>
@@ -392,6 +392,27 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>3/5</t>
+  </si>
+  <si>
+    <t>3/10</t>
+  </si>
+  <si>
+    <t>0/5</t>
+  </si>
+  <si>
+    <t>1/5</t>
+  </si>
+  <si>
+    <t>1/10</t>
+  </si>
+  <si>
+    <t>2/5</t>
+  </si>
+  <si>
+    <t>2/10</t>
   </si>
 </sst>
 </file>
@@ -6241,10 +6262,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77DBE236-4135-A849-993E-B5A600387A10}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6272,115 +6293,124 @@
       <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>30</v>
       </c>
       <c r="B2" s="1">
         <f>AVERAGE(C2:G2)</f>
-        <v>3.8461538461538464E-3</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1">
-        <f t="shared" ref="C2:E4" si="0">0/52</f>
+        <f>0/10</f>
         <v>0</v>
       </c>
       <c r="D2" s="1">
-        <f t="shared" si="0"/>
+        <f>0/10</f>
         <v>0</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" si="0"/>
+        <f>0/10</f>
         <v>0</v>
       </c>
       <c r="F2" s="1">
-        <f t="shared" ref="F2:F21" si="1">1/52</f>
-        <v>1.9230769230769232E-2</v>
+        <f>0/10</f>
+        <v>0</v>
       </c>
       <c r="G2" s="1">
-        <f t="shared" ref="G2:G21" si="2">0/52</f>
+        <f>0/10</f>
         <v>0</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>60</v>
       </c>
       <c r="B3" s="1">
-        <f t="shared" ref="B3:B21" si="3">AVERAGE(C3:G3)</f>
-        <v>3.8461538461538464E-3</v>
+        <f t="shared" ref="B3:B21" si="0">AVERAGE(C3:G3)</f>
+        <v>0.02</v>
       </c>
       <c r="C3" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C3:D9" si="1">0/10</f>
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>1/10</f>
+        <v>0.1</v>
       </c>
       <c r="F3" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>0/10</f>
+        <v>0</v>
       </c>
       <c r="G3" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="G3:G19" si="2">0/10</f>
         <v>0</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>90</v>
       </c>
       <c r="B4" s="1">
-        <f t="shared" si="3"/>
-        <v>3.8461538461538464E-3</v>
+        <f t="shared" si="0"/>
+        <v>0.04</v>
       </c>
       <c r="C4" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ref="E4:E21" si="3">1/10</f>
+        <v>0.1</v>
       </c>
       <c r="F4" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>1/10</f>
+        <v>0.1</v>
       </c>
       <c r="G4" s="1">
         <f t="shared" si="2"/>
@@ -6390,38 +6420,41 @@
         <v>4</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>120</v>
       </c>
       <c r="B5" s="1">
+        <f t="shared" si="0"/>
+        <v>0.04</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C5" s="1">
-        <f>1/52</f>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D5" s="1">
-        <f>1/52</f>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E5" s="1">
-        <f>1/52</f>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F5" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>1/10</f>
+        <v>0.1</v>
       </c>
       <c r="G5" s="1">
         <f t="shared" si="2"/>
@@ -6431,38 +6464,41 @@
         <v>5</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>150</v>
       </c>
       <c r="B6" s="1">
+        <f t="shared" si="0"/>
+        <v>0.04</v>
+      </c>
+      <c r="C6" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C6" s="1">
-        <f t="shared" ref="C6:E21" si="4">1/52</f>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E6" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F6" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>1/10</f>
+        <v>0.1</v>
       </c>
       <c r="G6" s="1">
         <f t="shared" si="2"/>
@@ -6472,38 +6508,41 @@
         <v>6</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>180</v>
       </c>
       <c r="B7" s="1">
+        <f t="shared" si="0"/>
+        <v>6.0000000000000012E-2</v>
+      </c>
+      <c r="C7" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C7" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D7" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E7" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>2/10</f>
+        <v>0.2</v>
       </c>
       <c r="G7" s="1">
         <f t="shared" si="2"/>
@@ -6513,270 +6552,273 @@
         <v>13</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>210</v>
       </c>
       <c r="B8" s="1">
+        <f t="shared" si="0"/>
+        <v>6.0000000000000012E-2</v>
+      </c>
+      <c r="C8" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C8" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D8" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E8" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F8" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>2/10</f>
+        <v>0.2</v>
       </c>
       <c r="G8" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>240</v>
       </c>
       <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="1">
+        <f>1/10</f>
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C9" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D9" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E9" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F9" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>3/10</f>
+        <v>0.3</v>
       </c>
       <c r="G9" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>270</v>
       </c>
       <c r="B10" s="1">
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
+      </c>
+      <c r="C10" s="1">
+        <f t="shared" ref="C10:D21" si="4">1/10</f>
+        <v>0.1</v>
+      </c>
+      <c r="D10" s="1">
+        <f>1/10</f>
+        <v>0.1</v>
+      </c>
+      <c r="E10" s="1">
         <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
-      </c>
-      <c r="C10" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="D10" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
-      </c>
-      <c r="E10" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F10" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" ref="F10:F21" si="5">3/10</f>
+        <v>0.3</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>300</v>
       </c>
       <c r="B11" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
       </c>
       <c r="C11" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E11" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F11" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G11" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>330</v>
       </c>
       <c r="B12" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
       </c>
       <c r="C12" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F12" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G12" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>360</v>
       </c>
       <c r="B13" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
       </c>
       <c r="C13" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F13" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G13" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>390</v>
       </c>
       <c r="B14" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
       </c>
       <c r="C14" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F14" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G14" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>420</v>
       </c>
       <c r="B15" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5384615384615385E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12000000000000002</v>
       </c>
       <c r="C15" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F15" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G15" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>450</v>
       </c>
       <c r="B16" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="C16" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f>3/10</f>
+        <v>0.3</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E16" s="1">
-        <f>2/52</f>
-        <v>3.8461538461538464E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F16" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G16" s="1">
         <f t="shared" si="2"/>
@@ -6788,24 +6830,24 @@
         <v>480</v>
       </c>
       <c r="B17" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="C17" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" ref="C17:C21" si="6">3/10</f>
+        <v>0.3</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E17" s="1">
-        <f t="shared" ref="E17:E21" si="5">2/52</f>
-        <v>3.8461538461538464E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F17" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="5"/>
+        <v>0.3</v>
       </c>
       <c r="G17" s="1">
         <f t="shared" si="2"/>
@@ -6817,24 +6859,24 @@
         <v>510</v>
       </c>
       <c r="B18" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="C18" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="6"/>
+        <v>0.3</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E18" s="1">
+        <f t="shared" si="3"/>
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="1">
         <f t="shared" si="5"/>
-        <v>3.8461538461538464E-2</v>
-      </c>
-      <c r="F18" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.3</v>
       </c>
       <c r="G18" s="1">
         <f t="shared" si="2"/>
@@ -6846,24 +6888,24 @@
         <v>540</v>
       </c>
       <c r="B19" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="C19" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="6"/>
+        <v>0.3</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E19" s="1">
+        <f t="shared" si="3"/>
+        <v>0.1</v>
+      </c>
+      <c r="F19" s="1">
         <f t="shared" si="5"/>
-        <v>3.8461538461538464E-2</v>
-      </c>
-      <c r="F19" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="1">
         <f t="shared" si="2"/>
@@ -6875,28 +6917,28 @@
         <v>570</v>
       </c>
       <c r="B20" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.18</v>
       </c>
       <c r="C20" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="6"/>
+        <v>0.3</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" si="5"/>
-        <v>3.8461538461538464E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.1</v>
       </c>
       <c r="F20" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <f>3/10</f>
+        <v>0.3</v>
       </c>
       <c r="G20" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>1/10</f>
+        <v>0.1</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -6904,32 +6946,33 @@
         <v>600</v>
       </c>
       <c r="B21" s="1">
-        <f t="shared" si="3"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.2</v>
       </c>
       <c r="C21" s="1">
-        <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <f t="shared" si="6"/>
+        <v>0.3</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" si="4"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E21" s="1">
+        <f t="shared" si="3"/>
+        <v>0.1</v>
+      </c>
+      <c r="F21" s="1">
         <f t="shared" si="5"/>
-        <v>3.8461538461538464E-2</v>
-      </c>
-      <c r="F21" s="1">
-        <f t="shared" si="1"/>
-        <v>1.9230769230769232E-2</v>
+        <v>0.3</v>
       </c>
       <c r="G21" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>2/10</f>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>